<commit_message>
Updated excel and util
</commit_message>
<xml_diff>
--- a/testData/testData.xlsx
+++ b/testData/testData.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
+    <sheet name="opportunities" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="125725"/>
   <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
   <si>
     <t>testCase</t>
   </si>
@@ -46,6 +47,51 @@
   </si>
   <si>
     <t>ValidCredentials</t>
+  </si>
+  <si>
+    <t>Create Opportunity</t>
+  </si>
+  <si>
+    <t>OpportunityName</t>
+  </si>
+  <si>
+    <t>Tester1</t>
+  </si>
+  <si>
+    <t>AccountName</t>
+  </si>
+  <si>
+    <t>Kaos Trading Ltd</t>
+  </si>
+  <si>
+    <t>OpportunityAmount</t>
+  </si>
+  <si>
+    <t>SalesStage</t>
+  </si>
+  <si>
+    <t>Prospecting</t>
+  </si>
+  <si>
+    <t>ExpectedCloseDate</t>
+  </si>
+  <si>
+    <t>BlankMandatoryfield</t>
+  </si>
+  <si>
+    <t>InvalidAmount</t>
+  </si>
+  <si>
+    <t>Test Opportunity</t>
+  </si>
+  <si>
+    <t>abc123</t>
+  </si>
+  <si>
+    <t>AccountSearch</t>
+  </si>
+  <si>
+    <t>Kaos</t>
   </si>
 </sst>
 </file>
@@ -81,8 +127,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -355,7 +402,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -416,4 +463,103 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>5000</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46387</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1">
+        <v>46387</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="1">
+        <v>46387</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Merge latest main into PW_Vara
</commit_message>
<xml_diff>
--- a/testData/testData.xlsx
+++ b/testData/testData.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11012"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pmano\PW_CRM\Playwright_Titans\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/varam/Desktop/NumpyNinja/Git_PW/Playwright_Titans/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6446C1A9-A3B8-47B6-BAC0-231D13F0B78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{343EA4D4-F299-6A40-82F4-9563D8878184}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="22260" windowHeight="12640" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
     <sheet name="opportunities" sheetId="2" r:id="rId2"/>
     <sheet name="LeadsData" sheetId="3" r:id="rId3"/>
-    <sheet name="Documents" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="125725"/>
   <extLst>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="88">
   <si>
     <t>testCase</t>
   </si>
@@ -292,24 +291,12 @@
   </si>
   <si>
     <t>Test lead for Robert Smith</t>
-  </si>
-  <si>
-    <t>PUBLISH DATE</t>
-  </si>
-  <si>
-    <t>REVISION</t>
-  </si>
-  <si>
-    <t>TC001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd;@"/>
-  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -368,14 +355,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -657,12 +643,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -673,7 +659,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -684,7 +670,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -695,7 +681,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -714,16 +700,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -743,7 +729,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -763,12 +749,12 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -788,7 +774,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -796,7 +782,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -813,9 +799,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB7CBB58-CC32-3442-AC7F-92AB77965A23}">
   <dimension ref="A1:V4"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:22" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -883,7 +869,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>45</v>
       </c>
@@ -951,7 +937,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>62</v>
       </c>
@@ -1019,7 +1005,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>75</v>
       </c>
@@ -1085,60 +1071,6 @@
       </c>
       <c r="V4" s="3" t="s">
         <v>87</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01E85675-CCBB-4BF0-940B-9BD2D2BEEE01}">
-  <dimension ref="A1:U2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.90625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B2" s="6">
-        <v>47026</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Meetings steps & Test data updated
</commit_message>
<xml_diff>
--- a/testData/testData.xlsx
+++ b/testData/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manga\PW1_Titans\Playwright_Titans\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{149CB0A3-319D-4906-A129-6365F197BDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A346FAD-543C-4627-9D97-66B82027BA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10800" yWindow="210" windowWidth="15795" windowHeight="15030" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
@@ -19,10 +19,21 @@
     <sheet name="meetings" sheetId="4" r:id="rId4"/>
     <sheet name="Quotes" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -32,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="98">
   <si>
     <t>testCase</t>
   </si>
@@ -298,15 +309,6 @@
     <t>Test lead for Robert Smith</t>
   </si>
   <si>
-    <t>Subject</t>
-  </si>
-  <si>
-    <t>CreateMeeting</t>
-  </si>
-  <si>
-    <t>Contract renewal1</t>
-  </si>
-  <si>
     <t>Title</t>
   </si>
   <si>
@@ -323,6 +325,18 @@
   </si>
   <si>
     <t>On Hold</t>
+  </si>
+  <si>
+    <t>Initial meeting</t>
+  </si>
+  <si>
+    <t>startDate</t>
+  </si>
+  <si>
+    <t>TC001</t>
+  </si>
+  <si>
+    <t>subject</t>
   </si>
 </sst>
 </file>
@@ -738,7 +752,7 @@
     <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -832,6 +846,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB7CBB58-CC32-3442-AC7F-92AB77965A23}">
   <dimension ref="A1:V4"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="31.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
@@ -1112,27 +1149,35 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11A1278E-4E8F-4C4D-B5F7-52E9C6CC17A7}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+      <c r="C1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>94</v>
+      </c>
+      <c r="C2" t="str">
+        <f ca="1">TEXT(TODAY()-1,"yyyy-mm-dd")</f>
+        <v>2026-10-04</v>
       </c>
     </row>
   </sheetData>
@@ -1156,24 +1201,24 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D2">
         <v>30</v>

</xml_diff>

<commit_message>
Meetings & Contact latest
</commit_message>
<xml_diff>
--- a/testData/testData.xlsx
+++ b/testData/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manga\PW1_Titans\Playwright_Titans\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A346FAD-543C-4627-9D97-66B82027BA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E831B8F-91D9-45BB-B457-071F03CFED47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="100">
   <si>
     <t>testCase</t>
   </si>
@@ -327,9 +327,6 @@
     <t>On Hold</t>
   </si>
   <si>
-    <t>Initial meeting</t>
-  </si>
-  <si>
     <t>startDate</t>
   </si>
   <si>
@@ -337,6 +334,15 @@
   </si>
   <si>
     <t>subject</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>Final negotiation</t>
+  </si>
+  <si>
+    <t>Contract final discussions</t>
   </si>
 </sst>
 </file>
@@ -1149,11 +1155,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11A1278E-4E8F-4C4D-B5F7-52E9C6CC17A7}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1162,22 +1168,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C2" t="str">
-        <f ca="1">TEXT(TODAY()-1,"yyyy-mm-dd")</f>
-        <v>2026-10-04</v>
+        <f ca="1">TEXT(TODAY(),"yyyy-mm-dd")</f>
+        <v>2026-10-05</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" t="str">
+        <f ca="1">TEXT(TODAY()-3,"yyyy-mm-dd")</f>
+        <v>2026-10-02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>